<commit_message>
Tracker: add Saela (applied, waiting) + founder outreach note
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TuhM6r1rkWffWN6sdrTeQ9
</commit_message>
<xml_diff>
--- a/job-search/remote-jobs-tracker.xlsx
+++ b/job-search/remote-jobs-tracker.xlsx
@@ -517,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -839,29 +839,66 @@
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="8" t="inlineStr">
+    <row r="12" ht="92" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Saela (Saela Sync)</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Data Analyst / Engineer</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Health-privacy SaaS (women's health AI)</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>Waiting</t>
+        </is>
+      </c>
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>Your strongest fit of the batch: SQL-first + you have founded and built your own product's data layer (MyFacit, promoted to a Founder experience entry here) + you manage AI agents daily. Also reached out to founder Maggie Lusk on LinkedIn. Gaps: they want 5+ yrs (you are ~2 + founder + internship - answer written to prove level, not apologise for years); TypeScript/React are 'some' + pairing offered; health domain new. Confirm remote/location. App answers drafted: why-company (with mission), pipeline, customer/marketing-data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="inlineStr">
         <is>
           <t>Legend:</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="9" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr">
         <is>
           <t>Rejected</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="10" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="10" t="inlineStr">
         <is>
           <t>Waiting</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="11" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="11" t="inlineStr">
         <is>
           <t>Outreach</t>
         </is>

</xml_diff>